<commit_message>
numerous files added and updated
</commit_message>
<xml_diff>
--- a/[SDLC] Scrum-Agile/Product Backlog & User Stories.xlsx
+++ b/[SDLC] Scrum-Agile/Product Backlog & User Stories.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\School &amp; Professional\~SNHU\CS 250 - Software Development Lifecycle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mathy\portfolio\[SDLC] Scrum-Agile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{856C3F54-74B0-48C4-A79A-FB78AFAB0135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F374DBAE-3B5A-4B4E-BEA8-B7BCD35D2B54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="4185" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="26715" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -597,7 +597,7 @@
     <col min="1" max="1" width="19" style="4" customWidth="1"/>
     <col min="2" max="2" width="24.85546875" style="4" customWidth="1"/>
     <col min="3" max="3" width="36.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.7109375" style="4" customWidth="1"/>
     <col min="6" max="6" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.7109375" style="4" bestFit="1" customWidth="1"/>

</xml_diff>